<commit_message>
📊 BIST Screener | 10.04.2026 16:30 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-10.xlsx
+++ b/data/bist_screener_2026-04-10.xlsx
@@ -25656,23 +25656,21 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>246.8</v>
+        <v>13.88</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.0221</v>
       </c>
       <c r="D580" s="5" t="n">
-        <v>8570</v>
-      </c>
-      <c r="E580" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>62600000</v>
+      </c>
+      <c r="E580" s="2" t="inlineStr"/>
       <c r="F580" s="3" t="n">
-        <v>44.96</v>
+        <v>55.01</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
@@ -25683,40 +25681,50 @@
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L580" s="2" t="inlineStr"/>
+      <c r="L580" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M580" s="2" t="inlineStr"/>
     </row>
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>2.97</v>
+        <v>3.38</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>0.0421</v>
+        <v>-0.0117</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>318550000</v>
-      </c>
-      <c r="E581" s="6" t="inlineStr"/>
+        <v>73620000</v>
+      </c>
+      <c r="E581" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F581" s="7" t="n">
-        <v>63.41</v>
+        <v>67.5</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
-      <c r="I581" s="6" t="inlineStr"/>
-      <c r="J581" s="6" t="inlineStr"/>
+      <c r="I581" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J581" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L581" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M581" s="6" t="inlineStr"/>
@@ -25724,56 +25732,60 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>37.9</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>0.0499</v>
+        <v>-0.0479</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>6340000</v>
-      </c>
-      <c r="E582" s="2" t="inlineStr"/>
+        <v>24330</v>
+      </c>
+      <c r="E582" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F582" s="3" t="n">
-        <v>57.82</v>
+        <v>33.09</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
-      <c r="I582" s="2" t="inlineStr"/>
-      <c r="J582" s="2" t="inlineStr"/>
+      <c r="I582" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J582" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L582" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L582" s="2" t="inlineStr"/>
       <c r="M582" s="2" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>23.54</v>
+        <v>3.67</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0208</v>
-      </c>
-      <c r="D583" s="9" t="n">
-        <v>16990000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
+        <v>0.0194</v>
+      </c>
+      <c r="D583" s="7" t="n">
+        <v>65930000.00000001</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F583" s="7" t="n">
-        <v>53.95</v>
+        <v>63.9</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25781,12 +25793,12 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25794,34 +25806,30 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>240.5</v>
+        <v>25.52</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0103</v>
-      </c>
-      <c r="D584" s="5" t="n">
-        <v>12900000</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="D584" s="2" t="inlineStr"/>
       <c r="E584" s="2" t="inlineStr"/>
-      <c r="F584" s="3" t="n">
-        <v>81.61</v>
-      </c>
+      <c r="F584" s="2" t="inlineStr"/>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
       <c r="J584" s="2" t="inlineStr"/>
       <c r="K584" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L584" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M584" s="2" t="inlineStr"/>
@@ -25829,40 +25837,34 @@
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>3.38</v>
+        <v>23.54</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>-0.0117</v>
+        <v>0.0208</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>73620000</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>16990000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>67.5</v>
+        <v>53.95</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J585" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I585" s="6" t="inlineStr"/>
+      <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25870,34 +25872,42 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>13.88</v>
+        <v>17.57</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0221</v>
+        <v>0.0104</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>62600000</v>
-      </c>
-      <c r="E586" s="2" t="inlineStr"/>
+        <v>12950000</v>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F586" s="3" t="n">
-        <v>55.01</v>
-      </c>
-      <c r="G586" s="2" t="inlineStr"/>
+        <v>50.28</v>
+      </c>
+      <c r="G586" s="3" t="n">
+        <v>166.07</v>
+      </c>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="2" t="inlineStr"/>
-      <c r="J586" s="2" t="inlineStr"/>
+      <c r="I586" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J586" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25905,21 +25915,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>17.01</v>
+        <v>240.5</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0</v>
+        <v>-0.0103</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>141990000</v>
+        <v>12900000</v>
       </c>
       <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>55.39</v>
+        <v>81.61</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25927,12 +25937,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25940,63 +25950,67 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>124.8</v>
+        <v>246.8</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.09960000000000001</v>
-      </c>
-      <c r="D588" s="2" t="inlineStr"/>
-      <c r="E588" s="2" t="inlineStr"/>
-      <c r="F588" s="2" t="inlineStr"/>
+        <v>0.04269999999999999</v>
+      </c>
+      <c r="D588" s="5" t="n">
+        <v>8570</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.2578</v>
+      </c>
+      <c r="F588" s="3" t="n">
+        <v>44.96</v>
+      </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr"/>
+      <c r="K588" s="2" t="inlineStr">
+        <is>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
       <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>3.99</v>
+        <v>190.6</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0992</v>
+        <v>0.0998</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>38830000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>14190000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>77.31</v>
+        <v>76.83</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26004,21 +26018,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>18.16</v>
+        <v>37.9</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.07519999999999999</v>
+        <v>0.0499</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>118530000</v>
+        <v>6340000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>88.15000000000001</v>
+        <v>57.82</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26026,12 +26040,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26039,21 +26053,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>42</v>
+        <v>17.01</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.0125</v>
+        <v>0</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>18620000</v>
+        <v>141990000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>57.33</v>
+        <v>55.39</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26061,12 +26075,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26111,40 +26125,34 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>154.2</v>
+        <v>42</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0265</v>
+        <v>0.0125</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>1170000</v>
-      </c>
-      <c r="E593" s="8" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>18620000</v>
+      </c>
+      <c r="E593" s="6" t="inlineStr"/>
       <c r="F593" s="7" t="n">
-        <v>71.59</v>
+        <v>57.33</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26152,94 +26160,94 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>33.26</v>
+        <v>10.5</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0692</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>5270000</v>
-      </c>
-      <c r="E594" s="2" t="inlineStr"/>
+        <v>281040</v>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F594" s="3" t="n">
-        <v>54.41</v>
+        <v>65.09</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>77.59999999999999</v>
+        <v>62.4</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0479</v>
+        <v>0.0331</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>24330</v>
+        <v>1040000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.58</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>33.09</v>
+        <v>58.43</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-9.409700000000001</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
       <c r="J595" s="8" t="n">
-        <v>-4.155</v>
+        <v>0.4139</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L595" s="6" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L595" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M595" s="6" t="inlineStr"/>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.31</v>
+        <v>124.8</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0145</v>
-      </c>
-      <c r="D596" s="5" t="n">
-        <v>14390000</v>
-      </c>
+        <v>-0.09960000000000001</v>
+      </c>
+      <c r="D596" s="2" t="inlineStr"/>
       <c r="E596" s="2" t="inlineStr"/>
-      <c r="F596" s="3" t="n">
-        <v>87.42</v>
-      </c>
+      <c r="F596" s="2" t="inlineStr"/>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
       <c r="I596" s="2" t="inlineStr"/>
@@ -26255,21 +26263,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>190.6</v>
+        <v>6.31</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0998</v>
+        <v>0.0145</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>14190000</v>
+        <v>14390000</v>
       </c>
       <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>76.83</v>
+        <v>87.42</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26277,34 +26285,32 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>75</v>
+        <v>28.04</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.09970000000000001</v>
+        <v>-0.0071</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>4440000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>9990000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>67.31</v>
+        <v>55.43</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26312,12 +26318,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26325,65 +26331,61 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>62.4</v>
+        <v>81.86</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0331</v>
+        <v>0.0004</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>1040000</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>12730000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>58.43</v>
+        <v>43.01</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="8" t="n">
-        <v>0.4139</v>
-      </c>
-      <c r="K599" s="6" t="inlineStr">
-        <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L599" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="J599" s="6" t="inlineStr"/>
+      <c r="K599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>25.52</v>
+        <v>2.97</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D600" s="2" t="inlineStr"/>
+        <v>0.0421</v>
+      </c>
+      <c r="D600" s="5" t="n">
+        <v>318550000</v>
+      </c>
       <c r="E600" s="2" t="inlineStr"/>
-      <c r="F600" s="2" t="inlineStr"/>
+      <c r="F600" s="3" t="n">
+        <v>63.41</v>
+      </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
       <c r="J600" s="2" t="inlineStr"/>
-      <c r="K600" s="2" t="inlineStr"/>
+      <c r="K600" s="2" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26391,28 +26393,32 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>3.67</v>
+        <v>3.99</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0194</v>
-      </c>
-      <c r="D601" s="7" t="n">
-        <v>65930000.00000001</v>
+        <v>0.0992</v>
+      </c>
+      <c r="D601" s="9" t="n">
+        <v>38830000</v>
       </c>
       <c r="E601" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.1672</v>
       </c>
       <c r="F601" s="7" t="n">
-        <v>63.9</v>
+        <v>77.31</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="6" t="inlineStr"/>
-      <c r="J601" s="6" t="inlineStr"/>
+      <c r="I601" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J601" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26420,7 +26426,7 @@
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26428,38 +26434,34 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>5.34</v>
+        <v>18.16</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.09949999999999999</v>
+        <v>0.07519999999999999</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>174330000</v>
-      </c>
-      <c r="E602" s="4" t="n">
-        <v>0.2478</v>
-      </c>
+        <v>118530000</v>
+      </c>
+      <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>13.18</v>
+        <v>88.15000000000001</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
-      <c r="I602" s="4" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26467,34 +26469,26 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>17.57</v>
+        <v>33.26</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0104</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>12950000</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>5270000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>50.28</v>
-      </c>
-      <c r="G603" s="7" t="n">
-        <v>166.07</v>
-      </c>
+        <v>54.41</v>
+      </c>
+      <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -26502,7 +26496,7 @@
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26510,38 +26504,40 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>2.76</v>
+        <v>154.2</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>0.0073</v>
+        <v>-0.0265</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>87790000</v>
+        <v>1170000</v>
       </c>
       <c r="E604" s="4" t="n">
-        <v>0.6898000000000001</v>
+        <v>0.1071</v>
       </c>
       <c r="F604" s="3" t="n">
-        <v>47.52</v>
+        <v>71.59</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
       <c r="J604" s="4" t="n">
-        <v>-2.0083</v>
+        <v>-0.4897</v>
       </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26549,50 +26545,60 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>81.86</v>
+        <v>2.76</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0004</v>
+        <v>0.0073</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>12730000</v>
-      </c>
-      <c r="E605" s="6" t="inlineStr"/>
+        <v>87790000</v>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>0.6898000000000001</v>
+      </c>
       <c r="F605" s="7" t="n">
-        <v>43.01</v>
+        <v>47.52</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
-      <c r="J605" s="6" t="inlineStr"/>
-      <c r="K605" s="6" t="inlineStr"/>
-      <c r="L605" s="6" t="inlineStr"/>
+      <c r="J605" s="8" t="n">
+        <v>-2.0083</v>
+      </c>
+      <c r="K605" s="6" t="inlineStr">
+        <is>
+          <t>Tüketici hizmetleri</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>28.04</v>
+        <v>75</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0071</v>
+        <v>0.09970000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>9990000</v>
-      </c>
-      <c r="E606" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>4440000</v>
+      </c>
+      <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>55.43</v>
+        <v>67.31</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26600,12 +26606,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26613,38 +26619,40 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>10.5</v>
+        <v>5.34</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>0.0692</v>
+        <v>-0.09949999999999999</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>281040</v>
+        <v>174330000</v>
       </c>
       <c r="E607" s="8" t="n">
-        <v>0.95</v>
+        <v>0.2478</v>
       </c>
       <c r="F607" s="7" t="n">
-        <v>65.09</v>
+        <v>13.18</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+        <v>-0.0005999999999999999</v>
+      </c>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr"/>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+        </is>
+      </c>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26669,7 +26677,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>10.04.2026 15:30</t>
+          <t>10.04.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 10.04.2026 18:04 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-10.xlsx
+++ b/data/bist_screener_2026-04-10.xlsx
@@ -25656,21 +25656,21 @@
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B580" s="3" t="n">
-        <v>13.88</v>
+        <v>33.26</v>
       </c>
       <c r="C580" s="4" t="n">
-        <v>0.0221</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="D580" s="5" t="n">
-        <v>62600000</v>
+        <v>5270000</v>
       </c>
       <c r="E580" s="2" t="inlineStr"/>
       <c r="F580" s="3" t="n">
-        <v>55.01</v>
+        <v>54.41</v>
       </c>
       <c r="G580" s="2" t="inlineStr"/>
       <c r="H580" s="2" t="inlineStr"/>
@@ -25678,12 +25678,12 @@
       <c r="J580" s="2" t="inlineStr"/>
       <c r="K580" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L580" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M580" s="2" t="inlineStr"/>
@@ -25691,40 +25691,34 @@
     <row r="581">
       <c r="A581" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B581" s="7" t="n">
-        <v>3.38</v>
+        <v>190.6</v>
       </c>
       <c r="C581" s="8" t="n">
-        <v>-0.0117</v>
+        <v>0.0998</v>
       </c>
       <c r="D581" s="9" t="n">
-        <v>73620000</v>
-      </c>
-      <c r="E581" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>14190000</v>
+      </c>
+      <c r="E581" s="6" t="inlineStr"/>
       <c r="F581" s="7" t="n">
-        <v>67.5</v>
+        <v>76.83</v>
       </c>
       <c r="G581" s="6" t="inlineStr"/>
       <c r="H581" s="6" t="inlineStr"/>
-      <c r="I581" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J581" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I581" s="6" t="inlineStr"/>
+      <c r="J581" s="6" t="inlineStr"/>
       <c r="K581" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L581" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M581" s="6" t="inlineStr"/>
@@ -25732,65 +25726,67 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>42</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>-0.0479</v>
+        <v>0.0125</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>24330</v>
-      </c>
-      <c r="E582" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>18620000</v>
+      </c>
+      <c r="E582" s="2" t="inlineStr"/>
       <c r="F582" s="3" t="n">
-        <v>33.09</v>
+        <v>57.33</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
-      <c r="I582" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J582" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I582" s="2" t="inlineStr"/>
+      <c r="J582" s="2" t="inlineStr"/>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L582" s="2" t="inlineStr"/>
+          <t>Elektronik teknoloji</t>
+        </is>
+      </c>
+      <c r="L582" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+        </is>
+      </c>
       <c r="M582" s="2" t="inlineStr"/>
     </row>
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>3.67</v>
+        <v>3.99</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0194</v>
-      </c>
-      <c r="D583" s="7" t="n">
-        <v>65930000.00000001</v>
+        <v>0.0992</v>
+      </c>
+      <c r="D583" s="9" t="n">
+        <v>38830000</v>
       </c>
       <c r="E583" s="8" t="n">
-        <v>0.8667</v>
+        <v>0.1672</v>
       </c>
       <c r="F583" s="7" t="n">
-        <v>63.9</v>
+        <v>77.31</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
-      <c r="I583" s="6" t="inlineStr"/>
-      <c r="J583" s="6" t="inlineStr"/>
+      <c r="I583" s="8" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J583" s="8" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K583" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -25798,7 +25794,7 @@
       </c>
       <c r="L583" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M583" s="6" t="inlineStr"/>
@@ -25806,18 +25802,22 @@
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>25.52</v>
+        <v>6.31</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D584" s="2" t="inlineStr"/>
+        <v>0.0145</v>
+      </c>
+      <c r="D584" s="5" t="n">
+        <v>14390000</v>
+      </c>
       <c r="E584" s="2" t="inlineStr"/>
-      <c r="F584" s="2" t="inlineStr"/>
+      <c r="F584" s="3" t="n">
+        <v>87.42</v>
+      </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
       <c r="I584" s="2" t="inlineStr"/>
@@ -25827,87 +25827,79 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L584" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
-        </is>
-      </c>
+      <c r="L584" s="2" t="inlineStr"/>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>23.54</v>
+        <v>10.5</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.0208</v>
+        <v>0.0692</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>16990000</v>
-      </c>
-      <c r="E585" s="6" t="inlineStr"/>
+        <v>281040</v>
+      </c>
+      <c r="E585" s="8" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F585" s="7" t="n">
-        <v>53.95</v>
+        <v>65.09</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="6" t="inlineStr"/>
-      <c r="J585" s="6" t="inlineStr"/>
+      <c r="I585" s="8" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J585" s="8" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L585" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L585" s="6" t="inlineStr"/>
       <c r="M585" s="6" t="inlineStr"/>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>17.57</v>
+        <v>28.04</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.0104</v>
+        <v>-0.0071</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>12950000</v>
+        <v>9990000</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.9246</v>
+        <v>0.2667</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>50.28</v>
-      </c>
-      <c r="G586" s="3" t="n">
-        <v>166.07</v>
-      </c>
+        <v>55.43</v>
+      </c>
+      <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
-      <c r="I586" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J586" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I586" s="2" t="inlineStr"/>
+      <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25915,34 +25907,42 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>240.5</v>
+        <v>17.57</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>-0.0103</v>
+        <v>0.0104</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>12900000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>12950000</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>81.61</v>
-      </c>
-      <c r="G587" s="6" t="inlineStr"/>
+        <v>50.28</v>
+      </c>
+      <c r="G587" s="7" t="n">
+        <v>166.07</v>
+      </c>
       <c r="H587" s="6" t="inlineStr"/>
-      <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="I587" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J587" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25950,54 +25950,48 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>246.8</v>
+        <v>81.86</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.04269999999999999</v>
+        <v>0.0004</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>8570</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>12730000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>44.96</v>
+        <v>43.01</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
       <c r="J588" s="2" t="inlineStr"/>
-      <c r="K588" s="2" t="inlineStr">
-        <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
+      <c r="K588" s="2" t="inlineStr"/>
       <c r="L588" s="2" t="inlineStr"/>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>190.6</v>
+        <v>23.54</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>0.0998</v>
+        <v>0.0208</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>14190000</v>
+        <v>16990000</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>76.83</v>
+        <v>53.95</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26005,12 +25999,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26018,34 +26012,38 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>37.9</v>
+        <v>5.34</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0499</v>
+        <v>-0.09949999999999999</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>6340000</v>
-      </c>
-      <c r="E590" s="2" t="inlineStr"/>
+        <v>174330000</v>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>0.2478</v>
+      </c>
       <c r="F590" s="3" t="n">
-        <v>57.82</v>
+        <v>13.18</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
-      <c r="I590" s="2" t="inlineStr"/>
+      <c r="I590" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26053,21 +26051,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>17.01</v>
+        <v>37.9</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0</v>
+        <v>0.0499</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>141990000</v>
+        <v>6340000</v>
       </c>
       <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>55.39</v>
+        <v>57.82</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26075,12 +26073,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26088,36 +26086,38 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>FENER</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>7.51</v>
+        <v>2.76</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0149</v>
+        <v>0.0073</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>12490000</v>
+        <v>87790000</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.28</v>
+        <v>0.6898000000000001</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>50.65</v>
+        <v>47.52</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="J592" s="4" t="n">
+        <v>-2.0083</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M592" s="2" t="inlineStr"/>
@@ -26125,34 +26125,30 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>42</v>
+        <v>25.52</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0.0125</v>
-      </c>
-      <c r="D593" s="9" t="n">
-        <v>18620000</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="D593" s="6" t="inlineStr"/>
       <c r="E593" s="6" t="inlineStr"/>
-      <c r="F593" s="7" t="n">
-        <v>57.33</v>
-      </c>
+      <c r="F593" s="6" t="inlineStr"/>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="6" t="inlineStr"/>
       <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26160,75 +26156,71 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>10.5</v>
+        <v>13.88</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0692</v>
+        <v>0.0221</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>281040</v>
-      </c>
-      <c r="E594" s="4" t="n">
-        <v>0.95</v>
-      </c>
+        <v>62600000</v>
+      </c>
+      <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>65.09</v>
+        <v>55.01</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J594" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I594" s="2" t="inlineStr"/>
+      <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
           <t>İşlenebilen endüstriler</t>
         </is>
       </c>
-      <c r="L594" s="2" t="inlineStr"/>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>62.4</v>
+        <v>3.67</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0331</v>
-      </c>
-      <c r="D595" s="9" t="n">
-        <v>1040000</v>
+        <v>0.0194</v>
+      </c>
+      <c r="D595" s="7" t="n">
+        <v>65930000.00000001</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.3695000000000001</v>
+        <v>0.8667</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>58.43</v>
+        <v>63.9</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="6" t="inlineStr"/>
-      <c r="J595" s="8" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26236,81 +26228,103 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>124.8</v>
+        <v>154.2</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.09960000000000001</v>
-      </c>
-      <c r="D596" s="2" t="inlineStr"/>
-      <c r="E596" s="2" t="inlineStr"/>
-      <c r="F596" s="2" t="inlineStr"/>
+        <v>-0.0265</v>
+      </c>
+      <c r="D596" s="5" t="n">
+        <v>1170000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.1071</v>
+      </c>
+      <c r="F596" s="3" t="n">
+        <v>71.59</v>
+      </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
-      <c r="I596" s="2" t="inlineStr"/>
-      <c r="J596" s="2" t="inlineStr"/>
+      <c r="I596" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J596" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L596" s="2" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L596" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>6.31</v>
+        <v>3.38</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0145</v>
+        <v>-0.0117</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>14390000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>73620000</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.7119</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>87.42</v>
+        <v>67.5</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-191.6342</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-0.8093</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>28.04</v>
+        <v>17.01</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0071</v>
+        <v>0</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>9990000</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>141990000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>55.43</v>
+        <v>55.39</v>
       </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
@@ -26318,12 +26332,12 @@
       <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26331,48 +26345,58 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>81.86</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0004</v>
+        <v>-0.0479</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>12730000</v>
-      </c>
-      <c r="E599" s="6" t="inlineStr"/>
+        <v>24330</v>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F599" s="7" t="n">
-        <v>43.01</v>
+        <v>33.09</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
-      <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="6" t="inlineStr"/>
-      <c r="K599" s="6" t="inlineStr"/>
+      <c r="I599" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J599" s="8" t="n">
+        <v>-4.155</v>
+      </c>
+      <c r="K599" s="6" t="inlineStr">
+        <is>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
       <c r="L599" s="6" t="inlineStr"/>
       <c r="M599" s="6" t="inlineStr"/>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>2.97</v>
+        <v>75</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0421</v>
+        <v>0.09970000000000001</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>318550000</v>
+        <v>4440000</v>
       </c>
       <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>63.41</v>
+        <v>67.31</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26380,12 +26404,12 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26393,32 +26417,26 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>3.99</v>
+        <v>2.97</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>0.0992</v>
+        <v>0.0421</v>
       </c>
       <c r="D601" s="9" t="n">
-        <v>38830000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>318550000</v>
+      </c>
+      <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>77.31</v>
+        <v>63.41</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26426,7 +26444,7 @@
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26434,21 +26452,23 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>SVGYO</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>18.16</v>
+        <v>7.51</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.07519999999999999</v>
+        <v>0.0149</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>118530000</v>
-      </c>
-      <c r="E602" s="2" t="inlineStr"/>
+        <v>12490000</v>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>0.28</v>
+      </c>
       <c r="F602" s="3" t="n">
-        <v>88.15000000000001</v>
+        <v>50.65</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
@@ -26461,7 +26481,7 @@
       </c>
       <c r="L602" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
         </is>
       </c>
       <c r="M602" s="2" t="inlineStr"/>
@@ -26469,21 +26489,23 @@
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>33.26</v>
+        <v>246.8</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.04269999999999999</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>5270000</v>
-      </c>
-      <c r="E603" s="6" t="inlineStr"/>
+        <v>8570</v>
+      </c>
+      <c r="E603" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F603" s="7" t="n">
-        <v>54.41</v>
+        <v>44.96</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26491,53 +26513,43 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr"/>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>154.2</v>
+        <v>240.5</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0265</v>
+        <v>-0.0103</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>1170000</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.1071</v>
-      </c>
+        <v>12900000</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>71.59</v>
+        <v>81.61</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="4" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J604" s="4" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I604" s="2" t="inlineStr"/>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L604" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M604" s="2" t="inlineStr"/>
@@ -26545,38 +26557,38 @@
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>FENER</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>2.76</v>
+        <v>62.4</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0073</v>
+        <v>0.0331</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>87790000</v>
+        <v>1040000</v>
       </c>
       <c r="E605" s="8" t="n">
-        <v>0.6898000000000001</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F605" s="7" t="n">
-        <v>47.52</v>
+        <v>58.43</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="8" t="n">
-        <v>-2.0083</v>
+        <v>0.4139</v>
       </c>
       <c r="K605" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L605" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M605" s="6" t="inlineStr"/>
@@ -26584,21 +26596,21 @@
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>SVGYO</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>75</v>
+        <v>18.16</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>0.09970000000000001</v>
+        <v>0.07519999999999999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>4440000</v>
+        <v>118530000</v>
       </c>
       <c r="E606" s="2" t="inlineStr"/>
       <c r="F606" s="3" t="n">
-        <v>67.31</v>
+        <v>88.15000000000001</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
@@ -26606,12 +26618,12 @@
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26619,40 +26631,28 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>5.34</v>
+        <v>124.8</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.09949999999999999</v>
-      </c>
-      <c r="D607" s="9" t="n">
-        <v>174330000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.2478</v>
-      </c>
-      <c r="F607" s="7" t="n">
-        <v>13.18</v>
-      </c>
+        <v>-0.09960000000000001</v>
+      </c>
+      <c r="D607" s="6" t="inlineStr"/>
+      <c r="E607" s="6" t="inlineStr"/>
+      <c r="F607" s="6" t="inlineStr"/>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
-        </is>
-      </c>
-      <c r="L607" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L607" s="6" t="inlineStr"/>
       <c r="M607" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26677,7 +26677,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>10.04.2026 16:30</t>
+          <t>10.04.2026 18:04</t>
         </is>
       </c>
     </row>

</xml_diff>